<commit_message>
rerun every stage under the new names, with intervals and a columns sheet
</commit_message>
<xml_diff>
--- a/02_HRvLR_groups/01_Design_Contrasts/c_data/design_contrasts.xlsx
+++ b/02_HRvLR_groups/01_Design_Contrasts/c_data/design_contrasts.xlsx
@@ -8,17 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="read_me" sheetId="1" r:id="rId1"/>
-    <sheet name="contrasts" sheetId="2" r:id="rId2"/>
-    <sheet name="correlation_strata" sheetId="3" r:id="rId3"/>
-    <sheet name="input_manifest" sheetId="4" r:id="rId4"/>
-    <sheet name="package_versions" sheetId="5" r:id="rId5"/>
+    <sheet name="columns" sheetId="2" r:id="rId2"/>
+    <sheet name="contrasts" sheetId="3" r:id="rId3"/>
+    <sheet name="correlation_strata" sheetId="4" r:id="rId4"/>
+    <sheet name="input_manifest" sheetId="5" r:id="rId5"/>
+    <sheet name="package_versions" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="173">
   <si>
     <t>sheet</t>
   </si>
@@ -26,6 +27,12 @@
     <t>holds</t>
   </si>
   <si>
+    <t>columns</t>
+  </si>
+  <si>
+    <t>Every column of every sheet below, with what it holds.</t>
+  </si>
+  <si>
     <t>contrasts</t>
   </si>
   <si>
@@ -50,15 +57,78 @@
     <t>Packages loaded at run time.</t>
   </si>
   <si>
+    <t>column</t>
+  </si>
+  <si>
+    <t>meaning</t>
+  </si>
+  <si>
     <t>definition</t>
   </si>
   <si>
+    <t>The contrast written as cell means.</t>
+  </si>
+  <si>
     <t>contrast</t>
   </si>
   <si>
+    <t>Comparison from the design: Training_&lt;group&gt; (T2 - T1), Acute_&lt;group&gt; (T3 - T2), Baseline/Trained/Acute_&lt;G1&gt;v&lt;G2&gt; (group difference at T1, T2, T3), Training/Acute_Interaction (difference in change).</t>
+  </si>
+  <si>
     <t>role</t>
   </si>
   <si>
+    <t>How the contrast is read: primary, secondary, descriptive, or floor (the baseline group difference).</t>
+  </si>
+  <si>
+    <t>level</t>
+  </si>
+  <si>
+    <t>Feature level: proteins, sets or modules.</t>
+  </si>
+  <si>
+    <t>correlation</t>
+  </si>
+  <si>
+    <t>Within-subject correlation estimated by duplicateCorrelation.</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>Name the script gives the file it read.</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>Path of the file read.</t>
+  </si>
+  <si>
+    <t>md5</t>
+  </si>
+  <si>
+    <t>MD5 checksum of the file read.</t>
+  </si>
+  <si>
+    <t>package</t>
+  </si>
+  <si>
+    <t>R package.</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>Package version.</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>Where the package came from.</t>
+  </si>
+  <si>
     <t>Training_HR = HR_T2 - HR_T1</t>
   </si>
   <si>
@@ -125,42 +195,18 @@
     <t>secondary</t>
   </si>
   <si>
-    <t>level</t>
-  </si>
-  <si>
-    <t>correlation</t>
-  </si>
-  <si>
     <t>within subject, from limpa's dpcDE fit with subject blocked</t>
   </si>
   <si>
-    <t>input</t>
-  </si>
-  <si>
-    <t>path</t>
-  </si>
-  <si>
-    <t>md5</t>
-  </si>
-  <si>
     <t>proteins</t>
   </si>
   <si>
-    <t>01_Trunk/03_Quantify/c_data/proteins.rds</t>
+    <t>01_Trunk/03_Quantification/c_data/proteins.rds</t>
   </si>
   <si>
     <t>34ef12f3ddbea70e6840925bab8692c5</t>
   </si>
   <si>
-    <t>package</t>
-  </si>
-  <si>
-    <t>version</t>
-  </si>
-  <si>
-    <t>source</t>
-  </si>
-  <si>
     <t>BiocGenerics</t>
   </si>
   <si>
@@ -179,6 +225,18 @@
     <t>CRAN (R 4.6.0)</t>
   </si>
   <si>
+    <t>bit</t>
+  </si>
+  <si>
+    <t>4.6.0</t>
+  </si>
+  <si>
+    <t>bit64</t>
+  </si>
+  <si>
+    <t>4.8.0</t>
+  </si>
+  <si>
     <t>circlize</t>
   </si>
   <si>
@@ -302,6 +360,12 @@
     <t>1.0.2</t>
   </si>
   <si>
+    <t>hms</t>
+  </si>
+  <si>
+    <t>1.1.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -374,6 +438,12 @@
     <t>1.1-3</t>
   </si>
   <si>
+    <t>readr</t>
+  </si>
+  <si>
+    <t>2.2.0</t>
+  </si>
+  <si>
     <t>renv</t>
   </si>
   <si>
@@ -446,10 +516,22 @@
     <t>tidyselect</t>
   </si>
   <si>
+    <t>tzdb</t>
+  </si>
+  <si>
+    <t>0.5.0</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
     <t>0.7.3</t>
+  </si>
+  <si>
+    <t>vroom</t>
+  </si>
+  <si>
+    <t>1.7.1</t>
   </si>
   <si>
     <t>writexl</t>
@@ -798,7 +880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1">
@@ -839,6 +921,14 @@
       </c>
       <c r="B5" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -848,23 +938,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -875,90 +965,112 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
         <v>20</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
         <v>22</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
         <v>25</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" t="s">
         <v>27</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
         <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>32</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C11" t="s">
         <v>33</v>
       </c>
-      <c r="C10" t="s">
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
         <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -968,23 +1080,117 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>37</v>
       </c>
-      <c r="B2">
-        <v>0.1702823336442219</v>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -994,29 +1200,23 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1">
+    <row r="1" spans="1:2" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
+        <v>58</v>
+      </c>
+      <c r="B2">
+        <v>0.1702823336442219</v>
       </c>
     </row>
   </sheetData>
@@ -1026,557 +1226,655 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="B11" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="B16" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="B18" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="B20" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="B21" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="B22" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="B23" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="B24" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="C24" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="B25" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="B26" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="C26" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="B27" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="C27" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="B28" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="B29" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="C29" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="B30" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="C30" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B31" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="C31" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="B32" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="B33" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="B34" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="C34" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="B35" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="C35" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B36" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="B37" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="C37" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="B38" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="C38" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="B39" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="C39" t="s">
-        <v>124</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="B40" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="C40" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B41" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="C41" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="B42" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="C42" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B43" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="C43" t="s">
-        <v>52</v>
+        <v>147</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="B44" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="C44" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="B45" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="C45" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="B46" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="C46" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="B47" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="C47" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="B48" t="s">
-        <v>76</v>
+        <v>157</v>
       </c>
       <c r="C48" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="B49" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="C49" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="B50" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
       <c r="C50" t="s">
-        <v>124</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
+        <v>162</v>
+      </c>
+      <c r="B51" t="s">
+        <v>163</v>
+      </c>
+      <c r="C51" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>164</v>
+      </c>
+      <c r="B52" t="s">
+        <v>95</v>
+      </c>
+      <c r="C52" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>165</v>
+      </c>
+      <c r="B53" t="s">
+        <v>166</v>
+      </c>
+      <c r="C53" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>167</v>
+      </c>
+      <c r="B54" t="s">
+        <v>168</v>
+      </c>
+      <c r="C54" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>169</v>
+      </c>
+      <c r="B55" t="s">
+        <v>170</v>
+      </c>
+      <c r="C55" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>171</v>
+      </c>
+      <c r="B56" t="s">
+        <v>172</v>
+      </c>
+      <c r="C56" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
decide who is compared first: one 02_Groups phase for HR/LR and the three clusterings
</commit_message>
<xml_diff>
--- a/02_HRvLR_groups/01_Design_Contrasts/c_data/design_contrasts.xlsx
+++ b/02_HRvLR_groups/01_Design_Contrasts/c_data/design_contrasts.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="182">
   <si>
     <t>sheet</t>
   </si>
@@ -207,6 +207,15 @@
     <t>34ef12f3ddbea70e6840925bab8692c5</t>
   </si>
   <si>
+    <t>groups</t>
+  </si>
+  <si>
+    <t>02_Groups/HRvLR/c_data/groups.rds</t>
+  </si>
+  <si>
+    <t>26f72a4304a4e04d6f21d4a12f304f9c</t>
+  </si>
+  <si>
     <t>BiocGenerics</t>
   </si>
   <si>
@@ -550,6 +559,12 @@
   </si>
   <si>
     <t>1.7.1</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -1238,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1261,6 +1276,17 @@
       </c>
       <c r="C2" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1270,7 +1296,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1286,629 +1312,640 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B10" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B16" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B17" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B18" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B19" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B20" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B21" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B22" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C22" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B23" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C23" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B24" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B25" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C25" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B26" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C26" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B27" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B28" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C28" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B29" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B30" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B31" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B32" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C32" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B34" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C34" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B35" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B36" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C36" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B37" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C37" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B38" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C38" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B39" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C39" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B40" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C40" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B41" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C41" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B42" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C42" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B43" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C43" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C44" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B45" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C45" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B46" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C46" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B47" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C47" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B48" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C48" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B49" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C49" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B50" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C50" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B51" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C51" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B52" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C52" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B53" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C53" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B54" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C54" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B55" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C55" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B56" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C56" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B57" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C57" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B58" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C58" t="s">
-        <v>67</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>180</v>
+      </c>
+      <c r="B59" t="s">
+        <v>181</v>
+      </c>
+      <c r="C59" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>